<commit_message>
chore: Dodaj skrypty pomocnicze i notatki MOPS
- Skrypty analizy danych (analyze, check, compare)
- Skrypty importu i czyszczenia (import-mops, clean, fix)
- Skrypty debugowania (debug-*, test-*)
- API endpointy MOPS (export, search)
- Strona MOPS (/app/mops)
- Zaktualizowane notatki w raw_dane

🤖 Generated with [Claude Code](https://claude.com/claude-code)

Co-Authored-By: Claude <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/raw_dane/malopolskie/Wykaz środowiskowych domów samopomocy(5).xlsx
+++ b/raw_dane/malopolskie/Wykaz środowiskowych domów samopomocy(5).xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/iwona/Documents/Projekty/kompas-seniora/raw_dane/malopolskie/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C14DE8CB-78AD-2845-A024-338FD405684E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{239ADF76-BF2B-544E-9CCA-CDD840A83148}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="760" windowWidth="28800" windowHeight="11320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="400" yWindow="2520" windowWidth="28680" windowHeight="15140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Arkusz1" sheetId="1" r:id="rId1"/>
@@ -5567,7 +5567,7 @@
         <v>385</v>
       </c>
     </row>
-    <row r="52" spans="1:11" ht="98" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:11" ht="84" x14ac:dyDescent="0.2">
       <c r="A52" s="4">
         <v>49</v>
       </c>

</xml_diff>